<commit_message>
large update: brownfield & restructuring
</commit_message>
<xml_diff>
--- a/data/GreenLab_Input_file.xlsx
+++ b/data/GreenLab_Input_file.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10921"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://aarhusuniversitet-my.sharepoint.com/personal/au731098_uni_au_dk/Documents/01_AU_Research/02_GreenLab/GLS II/GreenBubble_2/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://aarhusuniversitet-my.sharepoint.com/personal/au731098_uni_au_dk/Documents/01_AU_Research/09_GreenBubble/GLS_greenbubble/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{820E0913-7C8B-4D47-A4F2-F8681C44D888}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{158E70D0-1A56-9A42-877D-AFBBDBB6D741}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="13_ncr:1_{820E0913-7C8B-4D47-A4F2-F8681C44D888}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{47D9E9C7-862D-6144-AFF3-F82C48123512}"/>
   <bookViews>
     <workbookView xWindow="980" yWindow="760" windowWidth="29260" windowHeight="18880" activeTab="1" xr2:uid="{8A163641-094A-4E91-998B-38718FB15E01}"/>
   </bookViews>
@@ -222,10 +222,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Update GreenLab_Input_file.xlsx: methanolisation stream fluid CO2 pure -> H2
Overview_2 sheet, row 12: companion data fix for the methanolisation
bus0/efficiency rework (bus0 is now H2 in, was CO2 in).
</commit_message>
<xml_diff>
--- a/data/GreenLab_Input_file.xlsx
+++ b/data/GreenLab_Input_file.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10921"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://aarhusuniversitet-my.sharepoint.com/personal/au731098_uni_au_dk/Documents/01_AU_Research/09_GreenBubble/GLS_greenbubble/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/albal/Library/CloudStorage/OneDrive-DanmarksTekniskeUniversitet/01_DTU_research/01_Projects/02_greenbubble/GLS_greenbubble/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="13_ncr:1_{820E0913-7C8B-4D47-A4F2-F8681C44D888}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{47D9E9C7-862D-6144-AFF3-F82C48123512}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{132CBE01-DBF6-E94E-A825-87B7422A909C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="980" yWindow="760" windowWidth="29260" windowHeight="18880" activeTab="1" xr2:uid="{8A163641-094A-4E91-998B-38718FB15E01}"/>
+    <workbookView xWindow="980" yWindow="660" windowWidth="29260" windowHeight="17400" activeTab="1" xr2:uid="{8A163641-094A-4E91-998B-38718FB15E01}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="16" r:id="rId1"/>
@@ -826,7 +826,7 @@
         <v>9</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>